<commit_message>
updated SN74HCS08DR from library und reconnected the two parts. recreated outputjob files, but production was done with the zipped sources
</commit_message>
<xml_diff>
--- a/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/BOM_JLC/BOM_JLC_uz_per_wolfspeed_25kw_FM3_jlc_Rev04.xlsx
+++ b/Altium/Project Outputs for uz_per_wolfspeed_25kw_FM3/Rev04/BOM_JLC/BOM_JLC_uz_per_wolfspeed_25kw_FM3_jlc_Rev04.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_wolfspeed_25kw_fm3\Altium\Project Outputs for uz_per_wolfspeed_25kw_FM3\Rev04\BOM_JLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66B537EF-C4A3-470B-9243-A577872A7AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3520DE40-5F0D-45C4-88B4-DCE7E9F607BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EAC9EFF9-EC8B-4F2A-BDE2-5EE4534797F8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CD8CED93-5D71-4F24-AE18-BE4C896F2031}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC_uz_per_wolfspeed_25kw_F" sheetId="1" r:id="rId1"/>
@@ -428,19 +428,19 @@
     <t>SOIC127P600X175-14N</t>
   </si>
   <si>
-    <t>C2868021, [NoParam]</t>
-  </si>
-  <si>
-    <t>SN74LVC1G74DCUR</t>
+    <t>C2868021</t>
+  </si>
+  <si>
+    <t>SN74LVC1G74DCTR</t>
   </si>
   <si>
     <t>U14</t>
   </si>
   <si>
-    <t>VSSOP-8</t>
-  </si>
-  <si>
-    <t>C70285</t>
+    <t>MSOP-8</t>
+  </si>
+  <si>
+    <t>C840104</t>
   </si>
   <si>
     <t>R-RJ45R10P-B000</t>
@@ -857,7 +857,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E284D89-6964-44A1-9E27-6F952D42AC78}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55E5CEB4-42A0-4FE0-BAEC-1302CC0624F9}">
   <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>